<commit_message>
updates, tax bug fix
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2013" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48CAA3A6-F7F9-4842-8263-5CD87C0600B9}"/>
+  <xr:revisionPtr revIDLastSave="2044" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2369121-68EF-438B-AB4B-48CA83767D2E}"/>
   <bookViews>
-    <workbookView xWindow="-23025" yWindow="2145" windowWidth="21600" windowHeight="11100" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="2850" yWindow="1845" windowWidth="21600" windowHeight="11295" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2155" uniqueCount="789">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2172" uniqueCount="793">
   <si>
     <t>Durham</t>
   </si>
@@ -2405,6 +2405,18 @@
   </si>
   <si>
     <t>808base</t>
+  </si>
+  <si>
+    <t>H:\BRWM\PFAS - LD 1600\Sites\Cumberland\Gray Site (Christianson) (EGAD 29271)</t>
+  </si>
+  <si>
+    <t>Gray</t>
+  </si>
+  <si>
+    <t>L2656749-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no reporting </t>
   </si>
 </sst>
 </file>
@@ -6821,7 +6833,9 @@
       <c r="I117" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J117" s="4"/>
+      <c r="J117" s="4" t="s">
+        <v>783</v>
+      </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
@@ -6851,7 +6865,9 @@
       <c r="I118" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J118" s="4"/>
+      <c r="J118" s="4" t="s">
+        <v>783</v>
+      </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
@@ -6881,7 +6897,9 @@
       <c r="I119" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J119" s="4"/>
+      <c r="J119" s="4" t="s">
+        <v>783</v>
+      </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
@@ -6911,7 +6929,9 @@
       <c r="I120" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="J120" s="4"/>
+      <c r="J120" s="4" t="s">
+        <v>783</v>
+      </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
@@ -6937,7 +6957,9 @@
       <c r="A122" s="3" t="s">
         <v>588</v>
       </c>
-      <c r="B122" s="30"/>
+      <c r="B122" s="30" t="s">
+        <v>791</v>
+      </c>
       <c r="C122" s="3" t="s">
         <v>788</v>
       </c>
@@ -6947,11 +6969,24 @@
       <c r="E122" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F122" s="4"/>
-      <c r="G122" s="4"/>
-      <c r="H122" s="4"/>
-      <c r="I122" s="4"/>
-      <c r="J122" s="4"/>
+      <c r="F122" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G122" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H122" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I122" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="J122" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="K122" s="23" t="s">
+        <v>792</v>
+      </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123" s="3"/>
@@ -7250,7 +7285,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05C0069-E32D-47E3-8952-41BB91A7FDEB}">
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -10495,6 +10530,35 @@
       </c>
       <c r="H101" s="9" t="s">
         <v>786</v>
+      </c>
+    </row>
+    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>29271</v>
+      </c>
+      <c r="B102" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="C102" s="13" t="s">
+        <v>790</v>
+      </c>
+      <c r="D102" t="s">
+        <v>88</v>
+      </c>
+      <c r="E102" t="s">
+        <v>127</v>
+      </c>
+      <c r="F102" t="s">
+        <v>757</v>
+      </c>
+      <c r="H102" s="9" t="s">
+        <v>789</v>
+      </c>
+      <c r="K102">
+        <v>400597</v>
+      </c>
+      <c r="L102">
+        <v>4848180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change to data status calls and updates
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2044" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2369121-68EF-438B-AB4B-48CA83767D2E}"/>
+  <xr:revisionPtr revIDLastSave="2052" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDCDB360-9545-42E4-8BAC-1CBFF9E04CF3}"/>
   <bookViews>
-    <workbookView xWindow="2850" yWindow="1845" windowWidth="21600" windowHeight="11295" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2172" uniqueCount="793">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2178" uniqueCount="796">
   <si>
     <t>Durham</t>
   </si>
@@ -2417,6 +2417,15 @@
   </si>
   <si>
     <t xml:space="preserve">no reporting </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Souther Portland </t>
+  </si>
+  <si>
+    <t>Ahold Delhaize</t>
+  </si>
+  <si>
+    <t>Quinn</t>
   </si>
 </sst>
 </file>
@@ -2761,6 +2770,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -7285,7 +7298,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05C0069-E32D-47E3-8952-41BB91A7FDEB}">
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -10559,6 +10572,32 @@
       </c>
       <c r="L102">
         <v>4848180</v>
+      </c>
+    </row>
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>88</v>
+      </c>
+      <c r="B103" s="17" t="s">
+        <v>793</v>
+      </c>
+      <c r="C103" s="13" t="s">
+        <v>794</v>
+      </c>
+      <c r="D103" t="s">
+        <v>596</v>
+      </c>
+      <c r="E103" t="s">
+        <v>726</v>
+      </c>
+      <c r="F103" t="s">
+        <v>795</v>
+      </c>
+      <c r="K103">
+        <v>395950</v>
+      </c>
+      <c r="L103">
+        <v>4830753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
implimenting edd_compound.xlsx into compare_rags
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2063" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E4FC3BB-8A1A-4C25-A175-A9B6ABDF9E00}"/>
+  <xr:revisionPtr revIDLastSave="2074" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57EBF10D-1A7B-4961-BD3D-623461D58D43}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2187" uniqueCount="798">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2193" uniqueCount="801">
   <si>
     <t>Durham</t>
   </si>
@@ -2432,6 +2432,15 @@
   </si>
   <si>
     <t>L2656749-01D</t>
+  </si>
+  <si>
+    <t>New Glouster</t>
+  </si>
+  <si>
+    <t>H Johnston</t>
+  </si>
+  <si>
+    <t>H:\BRWM\PFAS - LD 1600\Sites\New Gloucester\H Johnston S-021541 New Gloucester</t>
   </si>
 </sst>
 </file>
@@ -7321,7 +7330,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05C0069-E32D-47E3-8952-41BB91A7FDEB}">
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -10608,7 +10617,7 @@
         <v>793</v>
       </c>
       <c r="D103" t="s">
-        <v>596</v>
+        <v>88</v>
       </c>
       <c r="E103" t="s">
         <v>726</v>
@@ -10621,6 +10630,35 @@
       </c>
       <c r="L103">
         <v>4830753</v>
+      </c>
+    </row>
+    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A104">
+        <v>29148</v>
+      </c>
+      <c r="B104" s="17" t="s">
+        <v>798</v>
+      </c>
+      <c r="C104" s="13" t="s">
+        <v>799</v>
+      </c>
+      <c r="D104" t="s">
+        <v>88</v>
+      </c>
+      <c r="E104" t="s">
+        <v>127</v>
+      </c>
+      <c r="F104" t="s">
+        <v>755</v>
+      </c>
+      <c r="I104" s="9" t="s">
+        <v>800</v>
+      </c>
+      <c r="K104">
+        <v>399074</v>
+      </c>
+      <c r="L104">
+        <v>4870081</v>
       </c>
     </row>
   </sheetData>
@@ -11689,12 +11727,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100125872C61801B94CBBE948BC6C9A2B9A" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="68502b0f0955ec7bc8f56677585c1c13">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="83b0043d-3627-4f29-99ea-ed882df73a05" xmlns:ns4="942c1815-1a1b-49ab-ae21-7a54e279a57b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7c7a778c7ed535cdadc2c6f960a471d8" ns3:_="" ns4:_="">
     <xsd:import namespace="83b0043d-3627-4f29-99ea-ed882df73a05"/>
@@ -11911,6 +11943,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80E629FC-C0A0-418E-A068-5110321EDDA0}">
   <ds:schemaRefs>
@@ -11920,15 +11958,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04CEB0DF-FBF6-4FAC-A4B6-1450ADA239FD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11945,4 +11974,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>